<commit_message>
docs: separate what the Gantt takes from the repository from what is a planning judgement
</commit_message>
<xml_diff>
--- a/docs/preliminary-report/plan/gantt.xlsx
+++ b/docs/preliminary-report/plan/gantt.xlsx
@@ -575,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -603,7 +603,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Project Gantt, September 2026 to June 2027  |  baseline of 24 October 2026  |  work packages derived from the repository (subprojects/*/README.md, docs/integration-contract.md)</t>
+          <t>Project Gantt, September 2026 to June 2027  |  baseline of 24 October 2026  |  work packages and interfaces from the repository, milestones from the FYP handbook, month spans are planning judgements</t>
         </is>
       </c>
     </row>
@@ -1358,8 +1358,15 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="20" t="inlineStr">
+        <is>
+          <t>Nothing in the repository records which month a work package runs: the bars are a baseline schedule derived from the deliverable dates, and may be moved without changing the plan's content.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A13:A16"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A36:M36"/>
@@ -1371,6 +1378,7 @@
     <mergeCell ref="A19:A21"/>
     <mergeCell ref="A22:A24"/>
     <mergeCell ref="A5:A12"/>
+    <mergeCell ref="A39:M39"/>
     <mergeCell ref="A38:M38"/>
     <mergeCell ref="A1:K1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs: make the Gantt this student's work plan, with other sub-projects as dependencies
</commit_message>
<xml_diff>
--- a/docs/preliminary-report/plan/gantt.xlsx
+++ b/docs/preliminary-report/plan/gantt.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Work plan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Group overview" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -71,7 +72,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -86,6 +87,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002F6F9F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BFBFBF"/>
       </patternFill>
     </fill>
     <fill>
@@ -168,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -191,12 +197,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -208,6 +212,10 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -575,7 +583,750 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:M34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="8.5" customWidth="1" min="3" max="3"/>
+    <col width="8.5" customWidth="1" min="4" max="4"/>
+    <col width="8.5" customWidth="1" min="5" max="5"/>
+    <col width="8.5" customWidth="1" min="6" max="6"/>
+    <col width="8.5" customWidth="1" min="7" max="7"/>
+    <col width="8.5" customWidth="1" min="8" max="8"/>
+    <col width="8.5" customWidth="1" min="9" max="9"/>
+    <col width="8.5" customWidth="1" min="10" max="10"/>
+    <col width="8.5" customWidth="1" min="11" max="11"/>
+    <col width="8.5" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sub-project 1: charging demand forecasting - work plan, September 2026 to June 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Xu Yuxuan, 2959485  |  baseline of 24 October 2026  |  main tasks from the FYP task book, sub-tasks per the handbook Gantt requirement, dependencies from the integration contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Sub-task</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Nov-26</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Dec-26</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Jan-27</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Feb-27</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Mar-27</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Apr-27</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>May-27</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Jun-27</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Status, 24 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>1  Collect and preprocess public charging datasets</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Dataset screening, licence check, dataset register</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n"/>
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="8" t="n"/>
+      <c r="H5" s="8" t="n"/>
+      <c r="I5" s="8" t="n"/>
+      <c r="J5" s="8" t="n"/>
+      <c r="K5" s="8" t="n"/>
+      <c r="L5" s="8" t="n"/>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="10" t="n"/>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Session-to-hourly pipeline with contract IO</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="8" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="8" t="n"/>
+      <c r="H6" s="8" t="n"/>
+      <c r="I6" s="8" t="n"/>
+      <c r="J6" s="8" t="n"/>
+      <c r="K6" s="8" t="n"/>
+      <c r="L6" s="8" t="n"/>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2  Analyse charging patterns and user behaviour</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Hourly profile, peak and trough, weekday structure</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="8" t="n"/>
+      <c r="H7" s="8" t="n"/>
+      <c r="I7" s="8" t="n"/>
+      <c r="J7" s="8" t="n"/>
+      <c r="K7" s="8" t="n"/>
+      <c r="L7" s="8" t="n"/>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="10" t="n"/>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Uncontrolled-charging baseline for the scheduler</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="8" t="n"/>
+      <c r="H8" s="8" t="n"/>
+      <c r="I8" s="8" t="n"/>
+      <c r="J8" s="8" t="n"/>
+      <c r="K8" s="8" t="n"/>
+      <c r="L8" s="8" t="n"/>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>3  Develop ML models for day-ahead demand</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Feature set: target-hour calendar, origin-anchored lags</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="8" t="n"/>
+      <c r="H9" s="8" t="n"/>
+      <c r="I9" s="8" t="n"/>
+      <c r="J9" s="8" t="n"/>
+      <c r="K9" s="8" t="n"/>
+      <c r="L9" s="8" t="n"/>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Seven-model comparison, 25-origin rolling backtest</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="8" t="n"/>
+      <c r="H10" s="8" t="n"/>
+      <c r="I10" s="8" t="n"/>
+      <c r="J10" s="8" t="n"/>
+      <c r="K10" s="8" t="n"/>
+      <c r="L10" s="8" t="n"/>
+      <c r="M10" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Cross-site validation on Palo Alto, no retuning</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="n"/>
+      <c r="H11" s="8" t="n"/>
+      <c r="I11" s="8" t="n"/>
+      <c r="J11" s="8" t="n"/>
+      <c r="K11" s="8" t="n"/>
+      <c r="L11" s="8" t="n"/>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>Done, 0.549 vs 0.670</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>4  Evaluate and compare accuracy</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Prediction intervals and coverage check</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="8" t="n"/>
+      <c r="H12" s="8" t="n"/>
+      <c r="I12" s="8" t="n"/>
+      <c r="J12" s="8" t="n"/>
+      <c r="K12" s="8" t="n"/>
+      <c r="L12" s="8" t="n"/>
+      <c r="M12" s="9" t="inlineStr">
+        <is>
+          <t>Done, 91.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>MAE, RMSE and MAPE with the zero-demand caveat</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="8" t="n"/>
+      <c r="H13" s="8" t="n"/>
+      <c r="I13" s="8" t="n"/>
+      <c r="J13" s="8" t="n"/>
+      <c r="K13" s="8" t="n"/>
+      <c r="L13" s="8" t="n"/>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>MAPE outstanding</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>5  Export forecasts in the agreed format</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Contract file plus metadata sidecar, wired into SP2</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="8" t="n"/>
+      <c r="H14" s="8" t="n"/>
+      <c r="I14" s="8" t="n"/>
+      <c r="J14" s="8" t="n"/>
+      <c r="K14" s="8" t="n"/>
+      <c r="L14" s="8" t="n"/>
+      <c r="M14" s="9" t="inlineStr">
+        <is>
+          <t>CSV + meta exist</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Interface freeze, contract v2</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="8" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="8" t="n"/>
+      <c r="I15" s="8" t="n"/>
+      <c r="J15" s="8" t="n"/>
+      <c r="K15" s="8" t="n"/>
+      <c r="L15" s="8" t="n"/>
+      <c r="M15" s="9" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Interim report and presentation</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="12" t="n"/>
+      <c r="G16" s="12" t="n"/>
+      <c r="H16" s="8" t="n"/>
+      <c r="I16" s="8" t="n"/>
+      <c r="J16" s="8" t="n"/>
+      <c r="K16" s="8" t="n"/>
+      <c r="L16" s="8" t="n"/>
+      <c r="M16" s="9" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Phase-3 evaluation support</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="8" t="n"/>
+      <c r="H17" s="12" t="n"/>
+      <c r="I17" s="12" t="n"/>
+      <c r="J17" s="12" t="n"/>
+      <c r="K17" s="8" t="n"/>
+      <c r="L17" s="8" t="n"/>
+      <c r="M17" s="9" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Dissertation and final poster</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="8" t="n"/>
+      <c r="F18" s="8" t="n"/>
+      <c r="G18" s="8" t="n"/>
+      <c r="H18" s="12" t="n"/>
+      <c r="I18" s="12" t="n"/>
+      <c r="J18" s="12" t="n"/>
+      <c r="K18" s="8" t="n"/>
+      <c r="L18" s="8" t="n"/>
+      <c r="M18" s="9" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Dependencies on other sub-projects (not this student's work)</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>SP5 cost and carbon baseline, the denominator of every saving</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="8" t="n"/>
+      <c r="G19" s="8" t="n"/>
+      <c r="H19" s="8" t="n"/>
+      <c r="I19" s="8" t="n"/>
+      <c r="J19" s="8" t="n"/>
+      <c r="K19" s="8" t="n"/>
+      <c r="L19" s="8" t="n"/>
+      <c r="M19" s="9" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>SP2 tariff table, needed before the scheduler is built</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="13" t="n"/>
+      <c r="E20" s="13" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
+      <c r="H20" s="8" t="n"/>
+      <c r="I20" s="8" t="n"/>
+      <c r="J20" s="8" t="n"/>
+      <c r="K20" s="8" t="n"/>
+      <c r="L20" s="8" t="n"/>
+      <c r="M20" s="9" t="inlineStr">
+        <is>
+          <t>External, issue #2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="10" t="n"/>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>SP4 dashboard wiring, consumes my contract file</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="8" t="n"/>
+      <c r="E21" s="8" t="n"/>
+      <c r="F21" s="13" t="n"/>
+      <c r="G21" s="13" t="n"/>
+      <c r="H21" s="8" t="n"/>
+      <c r="I21" s="8" t="n"/>
+      <c r="J21" s="8" t="n"/>
+      <c r="K21" s="8" t="n"/>
+      <c r="L21" s="8" t="n"/>
+      <c r="M21" s="9" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>Milestones (programme handbook)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>Project Specification &amp; Preliminary Report</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="8" t="n"/>
+      <c r="H24" s="8" t="n"/>
+      <c r="I24" s="8" t="n"/>
+      <c r="J24" s="8" t="n"/>
+      <c r="K24" s="8" t="n"/>
+      <c r="L24" s="8" t="n"/>
+      <c r="M24" s="17" t="inlineStr">
+        <is>
+          <t>30 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="8" t="n"/>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>Interim Report</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="8" t="n"/>
+      <c r="G25" s="16" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="n"/>
+      <c r="I25" s="8" t="n"/>
+      <c r="J25" s="8" t="n"/>
+      <c r="K25" s="8" t="n"/>
+      <c r="L25" s="8" t="n"/>
+      <c r="M25" s="17" t="inlineStr">
+        <is>
+          <t>8 Jan 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="8" t="n"/>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>Interim Presentation</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="8" t="n"/>
+      <c r="E26" s="8" t="n"/>
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="16" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="n"/>
+      <c r="I26" s="8" t="n"/>
+      <c r="J26" s="8" t="n"/>
+      <c r="K26" s="8" t="n"/>
+      <c r="L26" s="8" t="n"/>
+      <c r="M26" s="17" t="inlineStr">
+        <is>
+          <t>11-22 Jan 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>Final Poster</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="8" t="n"/>
+      <c r="E27" s="8" t="n"/>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="8" t="n"/>
+      <c r="H27" s="8" t="n"/>
+      <c r="I27" s="8" t="n"/>
+      <c r="J27" s="16" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="K27" s="8" t="n"/>
+      <c r="L27" s="8" t="n"/>
+      <c r="M27" s="17" t="inlineStr">
+        <is>
+          <t>19-21 Apr 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>Final Dissertation</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="8" t="n"/>
+      <c r="E28" s="8" t="n"/>
+      <c r="F28" s="8" t="n"/>
+      <c r="G28" s="8" t="n"/>
+      <c r="H28" s="8" t="n"/>
+      <c r="I28" s="8" t="n"/>
+      <c r="J28" s="16" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="K28" s="8" t="n"/>
+      <c r="L28" s="8" t="n"/>
+      <c r="M28" s="17" t="inlineStr">
+        <is>
+          <t>30 Apr 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="8" t="n"/>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>Project end (task book)</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="8" t="n"/>
+      <c r="F29" s="8" t="n"/>
+      <c r="G29" s="8" t="n"/>
+      <c r="H29" s="8" t="n"/>
+      <c r="I29" s="8" t="n"/>
+      <c r="J29" s="8" t="n"/>
+      <c r="K29" s="8" t="n"/>
+      <c r="L29" s="16" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="M29" s="17" t="inlineStr">
+        <is>
+          <t>1 Jul 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
+        <is>
+          <t>Reading the chart: a filled cell marks a month in which the sub-task is active.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr">
+        <is>
+          <t>Main tasks 1-5 are the five tasks named in the FYP task book; the rows beneath each are the sub-tasks the handbook asks for (p12, Gantt sheet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="18" t="inlineStr">
+        <is>
+          <t>Grey rows are other sub-projects. They are dependencies of this plan, not work reported here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>Month spans are planning judgements; only the status column records what exists on 24 October 2026.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A32:M32"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A31:M31"/>
+    <mergeCell ref="A33:M33"/>
+    <mergeCell ref="A34:M34"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A9:A11"/>
+  </mergeCells>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -603,19 +1354,19 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Project Gantt, September 2026 to June 2027  |  baseline of 24 October 2026  |  work packages and interfaces from the repository, milestones from the FYP handbook, month spans are planning judgements</t>
+          <t>Whole-platform view for group planning  |  baseline of 24 October 2026  |  work packages from subprojects/*/README.md, interfaces from docs/integration-contract.md</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Sub-project</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Work package</t>
+          <t>Sub-task</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -702,7 +1453,7 @@
       </c>
     </row>
     <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="10" t="n"/>
+      <c r="A6" s="11" t="n"/>
       <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Session-to-hourly demand pipeline</t>
@@ -725,7 +1476,7 @@
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="10" t="n"/>
+      <c r="A7" s="11" t="n"/>
       <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Features, direct multi-horizon models, 25-origin backtest</t>
@@ -748,7 +1499,7 @@
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="10" t="n"/>
+      <c r="A8" s="11" t="n"/>
       <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Cross-site validation, Palo Alto, no retuning</t>
@@ -771,7 +1522,7 @@
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="10" t="n"/>
+      <c r="A9" s="11" t="n"/>
       <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Contract export and integration with SP2/SP4/SP5</t>
@@ -794,7 +1545,7 @@
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="10" t="n"/>
+      <c r="A10" s="11" t="n"/>
       <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Interim report and presentation</t>
@@ -817,7 +1568,7 @@
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="10" t="n"/>
+      <c r="A11" s="11" t="n"/>
       <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Phase-3 evaluation support</t>
@@ -840,7 +1591,7 @@
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="11" t="n"/>
+      <c r="A12" s="10" t="n"/>
       <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Dissertation and final poster</t>
@@ -874,8 +1625,8 @@
         </is>
       </c>
       <c r="C13" s="8" t="n"/>
-      <c r="D13" s="12" t="n"/>
-      <c r="E13" s="12" t="n"/>
+      <c r="D13" s="19" t="n"/>
+      <c r="E13" s="19" t="n"/>
       <c r="F13" s="8" t="n"/>
       <c r="G13" s="8" t="n"/>
       <c r="H13" s="8" t="n"/>
@@ -890,7 +1641,7 @@
       </c>
     </row>
     <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="10" t="n"/>
+      <c r="A14" s="11" t="n"/>
       <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Scheduler build: LP / heuristic against valley filling</t>
@@ -898,8 +1649,8 @@
       </c>
       <c r="C14" s="8" t="n"/>
       <c r="D14" s="8" t="n"/>
-      <c r="E14" s="12" t="n"/>
-      <c r="F14" s="12" t="n"/>
+      <c r="E14" s="19" t="n"/>
+      <c r="F14" s="19" t="n"/>
       <c r="G14" s="8" t="n"/>
       <c r="H14" s="8" t="n"/>
       <c r="I14" s="8" t="n"/>
@@ -913,7 +1664,7 @@
       </c>
     </row>
     <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="10" t="n"/>
+      <c r="A15" s="11" t="n"/>
       <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Uncontrolled versus scheduled comparison</t>
@@ -922,8 +1673,8 @@
       <c r="C15" s="8" t="n"/>
       <c r="D15" s="8" t="n"/>
       <c r="E15" s="8" t="n"/>
-      <c r="F15" s="12" t="n"/>
-      <c r="G15" s="12" t="n"/>
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="19" t="n"/>
       <c r="H15" s="8" t="n"/>
       <c r="I15" s="8" t="n"/>
       <c r="J15" s="8" t="n"/>
@@ -936,7 +1687,7 @@
       </c>
     </row>
     <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="11" t="n"/>
+      <c r="A16" s="10" t="n"/>
       <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Phase-3 scenarios with SP1</t>
@@ -947,8 +1698,8 @@
       <c r="E16" s="8" t="n"/>
       <c r="F16" s="8" t="n"/>
       <c r="G16" s="8" t="n"/>
-      <c r="H16" s="12" t="n"/>
-      <c r="I16" s="12" t="n"/>
+      <c r="H16" s="19" t="n"/>
+      <c r="I16" s="19" t="n"/>
       <c r="J16" s="8" t="n"/>
       <c r="K16" s="8" t="n"/>
       <c r="L16" s="8" t="n"/>
@@ -973,8 +1724,8 @@
       <c r="D17" s="8" t="n"/>
       <c r="E17" s="8" t="n"/>
       <c r="F17" s="8" t="n"/>
-      <c r="G17" s="13" t="n"/>
-      <c r="H17" s="13" t="n"/>
+      <c r="G17" s="20" t="n"/>
+      <c r="H17" s="20" t="n"/>
       <c r="I17" s="8" t="n"/>
       <c r="J17" s="8" t="n"/>
       <c r="K17" s="8" t="n"/>
@@ -986,7 +1737,7 @@
       </c>
     </row>
     <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="11" t="n"/>
+      <c r="A18" s="10" t="n"/>
       <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Solar forecast module, ERA5 / NASA POWER</t>
@@ -998,8 +1749,8 @@
       <c r="F18" s="8" t="n"/>
       <c r="G18" s="8" t="n"/>
       <c r="H18" s="8" t="n"/>
-      <c r="I18" s="13" t="n"/>
-      <c r="J18" s="13" t="n"/>
+      <c r="I18" s="20" t="n"/>
+      <c r="J18" s="20" t="n"/>
       <c r="K18" s="8" t="n"/>
       <c r="L18" s="8" t="n"/>
       <c r="M18" s="9" t="inlineStr">
@@ -1019,8 +1770,8 @@
           <t>Initial dashboard script (on fork, not merged)</t>
         </is>
       </c>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="14" t="n"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="21" t="n"/>
       <c r="E19" s="8" t="n"/>
       <c r="F19" s="8" t="n"/>
       <c r="G19" s="8" t="n"/>
@@ -1036,7 +1787,7 @@
       </c>
     </row>
     <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="10" t="n"/>
+      <c r="A20" s="11" t="n"/>
       <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Wire the contract files, replace placeholder columns</t>
@@ -1045,8 +1796,8 @@
       <c r="C20" s="8" t="n"/>
       <c r="D20" s="8" t="n"/>
       <c r="E20" s="8" t="n"/>
-      <c r="F20" s="14" t="n"/>
-      <c r="G20" s="14" t="n"/>
+      <c r="F20" s="21" t="n"/>
+      <c r="G20" s="21" t="n"/>
       <c r="H20" s="8" t="n"/>
       <c r="I20" s="8" t="n"/>
       <c r="J20" s="8" t="n"/>
@@ -1059,7 +1810,7 @@
       </c>
     </row>
     <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="11" t="n"/>
+      <c r="A21" s="10" t="n"/>
       <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Views, integration test, reporting</t>
@@ -1071,8 +1822,8 @@
       <c r="F21" s="8" t="n"/>
       <c r="G21" s="8" t="n"/>
       <c r="H21" s="8" t="n"/>
-      <c r="I21" s="14" t="n"/>
-      <c r="J21" s="14" t="n"/>
+      <c r="I21" s="21" t="n"/>
+      <c r="J21" s="21" t="n"/>
       <c r="K21" s="8" t="n"/>
       <c r="L21" s="8" t="n"/>
       <c r="M21" s="9" t="inlineStr">
@@ -1093,8 +1844,8 @@
         </is>
       </c>
       <c r="C22" s="8" t="n"/>
-      <c r="D22" s="15" t="n"/>
-      <c r="E22" s="15" t="n"/>
+      <c r="D22" s="22" t="n"/>
+      <c r="E22" s="22" t="n"/>
       <c r="F22" s="8" t="n"/>
       <c r="G22" s="8" t="n"/>
       <c r="H22" s="8" t="n"/>
@@ -1109,7 +1860,7 @@
       </c>
     </row>
     <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="10" t="n"/>
+      <c r="A23" s="11" t="n"/>
       <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Savings, emissions and benchmarking</t>
@@ -1120,9 +1871,9 @@
       <c r="E23" s="8" t="n"/>
       <c r="F23" s="8" t="n"/>
       <c r="G23" s="8" t="n"/>
-      <c r="H23" s="15" t="n"/>
-      <c r="I23" s="15" t="n"/>
-      <c r="J23" s="15" t="n"/>
+      <c r="H23" s="22" t="n"/>
+      <c r="I23" s="22" t="n"/>
+      <c r="J23" s="22" t="n"/>
       <c r="K23" s="8" t="n"/>
       <c r="L23" s="8" t="n"/>
       <c r="M23" s="9" t="inlineStr">
@@ -1132,7 +1883,7 @@
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="11" t="n"/>
+      <c r="A24" s="10" t="n"/>
       <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Final assessment report for the dashboard</t>
@@ -1145,8 +1896,8 @@
       <c r="G24" s="8" t="n"/>
       <c r="H24" s="8" t="n"/>
       <c r="I24" s="8" t="n"/>
-      <c r="J24" s="15" t="n"/>
-      <c r="K24" s="15" t="n"/>
+      <c r="J24" s="22" t="n"/>
+      <c r="K24" s="22" t="n"/>
       <c r="L24" s="8" t="n"/>
       <c r="M24" s="9" t="inlineStr">
         <is>
@@ -1155,7 +1906,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Milestones (programme handbook)</t>
         </is>
@@ -1163,13 +1914,13 @@
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="8" t="n"/>
-      <c r="B27" s="17" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>Project Specification &amp; Preliminary Report</t>
         </is>
       </c>
       <c r="C27" s="8" t="n"/>
-      <c r="D27" s="18" t="inlineStr">
+      <c r="D27" s="16" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
@@ -1182,7 +1933,7 @@
       <c r="J27" s="8" t="n"/>
       <c r="K27" s="8" t="n"/>
       <c r="L27" s="8" t="n"/>
-      <c r="M27" s="19" t="inlineStr">
+      <c r="M27" s="17" t="inlineStr">
         <is>
           <t>30 Oct 2026</t>
         </is>
@@ -1190,7 +1941,7 @@
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="8" t="n"/>
-      <c r="B28" s="17" t="inlineStr">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>Interim Report</t>
         </is>
@@ -1199,7 +1950,7 @@
       <c r="D28" s="8" t="n"/>
       <c r="E28" s="8" t="n"/>
       <c r="F28" s="8" t="n"/>
-      <c r="G28" s="18" t="inlineStr">
+      <c r="G28" s="16" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
@@ -1209,7 +1960,7 @@
       <c r="J28" s="8" t="n"/>
       <c r="K28" s="8" t="n"/>
       <c r="L28" s="8" t="n"/>
-      <c r="M28" s="19" t="inlineStr">
+      <c r="M28" s="17" t="inlineStr">
         <is>
           <t>8 Jan 2027</t>
         </is>
@@ -1217,7 +1968,7 @@
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="8" t="n"/>
-      <c r="B29" s="17" t="inlineStr">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>Interim Presentation</t>
         </is>
@@ -1226,7 +1977,7 @@
       <c r="D29" s="8" t="n"/>
       <c r="E29" s="8" t="n"/>
       <c r="F29" s="8" t="n"/>
-      <c r="G29" s="18" t="inlineStr">
+      <c r="G29" s="16" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
@@ -1236,7 +1987,7 @@
       <c r="J29" s="8" t="n"/>
       <c r="K29" s="8" t="n"/>
       <c r="L29" s="8" t="n"/>
-      <c r="M29" s="19" t="inlineStr">
+      <c r="M29" s="17" t="inlineStr">
         <is>
           <t>11-22 Jan 2027</t>
         </is>
@@ -1244,7 +1995,7 @@
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="8" t="n"/>
-      <c r="B30" s="17" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>Final Poster</t>
         </is>
@@ -1256,14 +2007,14 @@
       <c r="G30" s="8" t="n"/>
       <c r="H30" s="8" t="n"/>
       <c r="I30" s="8" t="n"/>
-      <c r="J30" s="18" t="inlineStr">
+      <c r="J30" s="16" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
       </c>
       <c r="K30" s="8" t="n"/>
       <c r="L30" s="8" t="n"/>
-      <c r="M30" s="19" t="inlineStr">
+      <c r="M30" s="17" t="inlineStr">
         <is>
           <t>19-21 Apr 2027</t>
         </is>
@@ -1271,7 +2022,7 @@
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="8" t="n"/>
-      <c r="B31" s="17" t="inlineStr">
+      <c r="B31" s="15" t="inlineStr">
         <is>
           <t>Final Dissertation</t>
         </is>
@@ -1283,14 +2034,14 @@
       <c r="G31" s="8" t="n"/>
       <c r="H31" s="8" t="n"/>
       <c r="I31" s="8" t="n"/>
-      <c r="J31" s="18" t="inlineStr">
+      <c r="J31" s="16" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
       </c>
       <c r="K31" s="8" t="n"/>
       <c r="L31" s="8" t="n"/>
-      <c r="M31" s="19" t="inlineStr">
+      <c r="M31" s="17" t="inlineStr">
         <is>
           <t>30 Apr 2027</t>
         </is>
@@ -1298,7 +2049,7 @@
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="8" t="n"/>
-      <c r="B32" s="17" t="inlineStr">
+      <c r="B32" s="15" t="inlineStr">
         <is>
           <t>Project end (task book)</t>
         </is>
@@ -1312,61 +2063,54 @@
       <c r="I32" s="8" t="n"/>
       <c r="J32" s="8" t="n"/>
       <c r="K32" s="8" t="n"/>
-      <c r="L32" s="18" t="inlineStr">
+      <c r="L32" s="16" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
       </c>
-      <c r="M32" s="19" t="inlineStr">
+      <c r="M32" s="17" t="inlineStr">
         <is>
           <t>1 Jul 2027</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="20" t="inlineStr">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>Reading the chart: a filled cell marks a month in which the work package is active.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="20" t="inlineStr">
+      <c r="A35" s="18" t="inlineStr">
         <is>
           <t>Owners are taken from the sub-project READMEs; SP3 is still unallocated and is shown as a risk.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="20" t="inlineStr">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>SP1 bars marked Done are evidenced by the merged pipeline, the 77 passing tests and the Phase-1 report.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="20" t="inlineStr">
+      <c r="A37" s="18" t="inlineStr">
         <is>
           <t>SP4's September bar records an initial dashboard script that exists only on a fork, not in the main repository.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="20" t="inlineStr">
-        <is>
-          <t>Consumers and producers of every arrow are fixed in docs/integration-contract.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="20" t="inlineStr">
-        <is>
-          <t>Nothing in the repository records which month a work package runs: the bars are a baseline schedule derived from the deliverable dates, and may be moved without changing the plan's content.</t>
+      <c r="A38" s="18" t="inlineStr">
+        <is>
+          <t>Month spans are planning judgements; only the status column records what exists on 24 October 2026.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="13">
     <mergeCell ref="A13:A16"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A36:M36"/>
@@ -1378,7 +2122,6 @@
     <mergeCell ref="A19:A21"/>
     <mergeCell ref="A22:A24"/>
     <mergeCell ref="A5:A12"/>
-    <mergeCell ref="A39:M39"/>
     <mergeCell ref="A38:M38"/>
     <mergeCell ref="A1:K1"/>
   </mergeCells>
@@ -1387,13 +2130,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1402,119 +2145,136 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="21" t="inlineStr">
+      <c r="B1" s="23" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="C1" s="21" t="inlineStr">
+      <c r="C1" s="23" t="inlineStr">
         <is>
           <t>Weight / note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>30 Oct 2026</t>
         </is>
       </c>
-      <c r="B2" s="22" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>Project Specification &amp; Preliminary Report</t>
         </is>
       </c>
-      <c r="C2" s="22" t="inlineStr">
+      <c r="C2" s="24" t="inlineStr">
         <is>
           <t>10% of the final mark</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="22" t="inlineStr">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>21 Nov 2026</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>Supervisor grades the above</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="inlineStr">
+        <is>
+          <t>administrative deadline</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>8 Jan 2027</t>
         </is>
       </c>
-      <c r="B3" s="22" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>Interim Report</t>
         </is>
       </c>
-      <c r="C3" s="22" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>11-22 Jan 2027</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Interim Presentation</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>window set by the school</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>19-21 Apr 2027</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Final Poster</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="22" t="inlineStr">
-        <is>
-          <t>11-22 Jan 2027</t>
-        </is>
-      </c>
-      <c r="B4" s="22" t="inlineStr">
-        <is>
-          <t>Interim Presentation</t>
-        </is>
-      </c>
-      <c r="C4" s="22" t="inlineStr">
-        <is>
-          <t>window set by the school</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="22" t="inlineStr">
-        <is>
-          <t>19-21 Apr 2027</t>
-        </is>
-      </c>
-      <c r="B5" s="22" t="inlineStr">
-        <is>
-          <t>Final Poster</t>
-        </is>
-      </c>
-      <c r="C5" s="22" t="inlineStr">
-        <is>
-          <t>assessed</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>30 Apr 2027</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Final Dissertation</t>
         </is>
       </c>
-      <c r="C6" s="22" t="inlineStr">
-        <is>
-          <t>main submission</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>40%, main submission</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>1 Jul 2027</t>
         </is>
       </c>
-      <c r="B7" s="22" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>Project end</t>
         </is>
       </c>
-      <c r="C7" s="22" t="inlineStr">
+      <c r="C8" s="24" t="inlineStr">
         <is>
           <t>task-book end date</t>
         </is>

</xml_diff>